<commit_message>
Mobile UX: fit the full learning loop in the first fold
Redesign the practice webapp so a phone shows the whole loop (prompt, 4 options, answer feedback) without scrolling. Pin Lanjut to the viewport bottom while answered so continuing never needs a scroll; collapse the two un-picked distractors on answer so the reveal rises into the fold. Tuck the word-by-word breakdown behind a Rincian kata toggle. Density pass on header, stats, card, and options; the app container fades in (no lingering transform) so the pinned button stays viewport-relative.

Verified at 390x844: question state needs zero scroll (worst case last option at 598px, footer 665px); answer state keeps feedback visible with the action pinned. Desktop unaffected. Also bundles in-progress vocab data (db, xlsx, example batches 10-11).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vocabulary-tracker.xlsx
+++ b/vocabulary-tracker.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H543"/>
+  <dimension ref="A1:H581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22182,6 +22182,1374 @@
       <c r="H543" s="2" t="inlineStr">
         <is>
           <t>Memperkuat/mengulang kata sebelumnya. Contoh: มากๆ</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>นาฬิกา</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>naaliikaa</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr"/>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>jam (benda)</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F544" t="n">
+        <v>1</v>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>kata umum untuk jam dinding/tangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>ตี</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>tii</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr"/>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>jam dini hari (1-5)</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F545" t="n">
+        <v>1</v>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>ตีหนึ่ง = jam 1 pagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>โมงเช้า</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>moong cháo</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr"/>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>jam pagi (6-11)</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F546" t="n">
+        <v>3</v>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>หกโมงเช้า = jam 6 pagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>เที่ยง</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>thîiang</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr"/>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>tengah hari</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>1</v>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>jam 12.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>บ่าย</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>bàai</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr"/>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>sore (13-15)</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>1</v>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>บ่ายสอง = jam 2 siang</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>ทุ่ม</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>thûm</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr"/>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>malam (18-23)</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>1</v>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>หนึ่งทุ่ม = jam 7 malam</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>เที่ยงคืน</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>thîiang khuun</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr"/>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>tengah malam</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>1</v>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>jam 00.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>ครึ่ง</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>khrûeng</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr"/>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>setengah</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F551" t="n">
+        <v>4</v>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>สิบโมงครึ่ง = jam 10.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>ตอนเช้า</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>toon cháo</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr"/>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>pagi hari</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F552" t="n">
+        <v>2</v>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>ตอน = pada/waktu</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>กี่โมง</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>kìi moong</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr"/>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>jam berapa</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Waktu</t>
+        </is>
+      </c>
+      <c r="F553" t="n">
+        <v>3</v>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>pola tanya waktu</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>ดีกว่า</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>dii kwàa</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr"/>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>lebih baik</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Perbandingan</t>
+        </is>
+      </c>
+      <c r="F554" t="n">
+        <v>1</v>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>กว่า = penanda komparatif</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>ง่าย</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>ngâai</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr"/>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>mudah</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Sifat</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>3</v>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>ง่ายกว่า = lebih mudah</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>ยาก</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>yâak</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr"/>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>sulit</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Sifat</t>
+        </is>
+      </c>
+      <c r="F556" t="n">
+        <v>1</v>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>antonim ง่าย</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>เสถียร</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>sàthiian</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr"/>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>stabil</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Sifat</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>1</v>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>ไม่เสถียร = tidak stabil</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>ทุกวัน</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>thúk wan</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr"/>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>setiap hari</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="F558" t="n">
+        <v>2</v>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>ทุกวันทุกวัน = tiap hari terus!</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>บางวัน</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>baang wan</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr"/>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>kadang suatu hari</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="F559" t="n">
+        <v>2</v>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>beda dari บางครั้ง</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>บางครั้ง</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>baang khráng</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr"/>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>kadang-kadang</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>3</v>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>lebih formal dari บางที</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>หลังจาก</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>lǎng jàak</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr"/>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>setelah/sesudah</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Konjungsi</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>5</v>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>หลัง saja = versi santai</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>ต่อ</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>tòo</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr"/>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>lanjut/terus</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Konjungsi</t>
+        </is>
+      </c>
+      <c r="F562" t="n">
+        <v>4</v>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>ทำต่อ, ไปต่อ, อ่านต่อ</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>ตื่นนอน</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>tùuen noon</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr"/>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>bangun tidur</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F563" t="n">
+        <v>1</v>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>ตื่น = bangun, นอน = tidur</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>เริ่มงาน</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>rôoem ngaan</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr"/>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>mulai kerja</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F564" t="n">
+        <v>4</v>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>เริ่ม = mulai</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>เปิด</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>pôoet</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr"/>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>nyalakan/buka</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>2</v>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>เปิดคอม = nyalakan komputer</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>อ่าน</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>àan</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr"/>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>membaca</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>2</v>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>อ่านอีเมล = baca email</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>ส่ง</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>sòng</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr"/>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>mengirim/menyerahkan</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>3</v>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>ส่งงาน = kumpul tugas</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>เช็ค</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>chék</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr"/>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>mengecek</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F568" t="n">
+        <v>3</v>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>เช็คอีเมล, เช็คเอกสาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>ทิ้ง</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>thîng</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr"/>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>buang/abaikan</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Kegiatan</t>
+        </is>
+      </c>
+      <c r="F569" t="n">
+        <v>1</v>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>ทิ้งไว้ก่อน = skip dulu</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>ทีม</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>thiim</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr"/>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Orang</t>
+        </is>
+      </c>
+      <c r="F570" t="n">
+        <v>2</v>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>kata serapan Inggris</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>เอกสาร</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>èkkasǎan</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr"/>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>dokumen</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F571" t="n">
+        <v>6</v>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>kata formal kantor</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>อีเมล</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>iimeel</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr"/>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F572" t="n">
+        <v>6</v>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>kata serapan Inggris</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>คอมพิวเตอร์</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>khoomphiwtôoe</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr"/>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>komputer</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>2</v>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>versi pendek: คอม</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>บัญชี</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>banchii</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr"/>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>akuntansi</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F574" t="n">
+        <v>2</v>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>นักบัญชี = akuntan</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>หน้าที่</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>nâa thîi</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr"/>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>tugas/tanggung jawab</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F575" t="n">
+        <v>2</v>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>job desc dalam konteks kantor</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>ความคิด</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>khwaam khít</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr"/>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>pemikiran/ide</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F576" t="n">
+        <v>1</v>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>ความ = prefiks benda abstrak</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>ข้าวกลางวัน</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>khâao glaang wan</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr"/>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>makan siang</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Benda</t>
+        </is>
+      </c>
+      <c r="F577" t="n">
+        <v>1</v>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>ข้าวเช้า = sarapan, ข้าวเย็น = makan malam</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>ควร</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>khuuan</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr"/>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>seharusnya</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Modal</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>2</v>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>lebih lunak dari ต้อง</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>ไม่ให้</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>mâi hâi</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr"/>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>tidak izinkan</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Modal</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>2</v>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>ไม่ให้ไป = tidak boleh pergi</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>แต่ละคน</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>tàe là khon</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr"/>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>setiap orang</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Ekspresi</t>
+        </is>
+      </c>
+      <c r="F580" t="n">
+        <v>1</v>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>แต่ละ = setiap/masing-masing</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>ไม่เหมือนกัน</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>mâi mǔuean gan</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr"/>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>berbeda-beda</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Ekspresi</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>1</v>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>เหมือนกัน = sama satu sama lain</t>
         </is>
       </c>
     </row>

</xml_diff>